<commit_message>
Add explicit loop pattern MCQs
</commit_message>
<xml_diff>
--- a/content/Question Bank/MCQ/Python/Unit 4 - Looping/Unit 4 - Looping - MCQ.xlsx
+++ b/content/Question Bank/MCQ/Python/Unit 4 - Looping/Unit 4 - Looping - MCQ.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Python - MCQ - 4" sheetId="1" r:id="R26dcf14b7619437b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Python - MCQ - 4" sheetId="1" r:id="Rcbbd4f1d44064ab6"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -1866,17 +1866,17 @@
         <x:v>Python - MCQ - 4.2.15</x:v>
       </x:c>
       <x:c r="B26" t="str">
-        <x:v>A status board builds two rows:
-```python
-for row in range(2):
-    for column in range(3):
-        print(row, end="")
+        <x:v>A number pattern should grow by one digit on each row:
+```python
+for row in range(1, 4):
+    for number in range(1, row + 1):
+        print(number, end="")
     print()
 ```
-Which layout appears?</x:v>
+Which pattern is printed?</x:v>
       </x:c>
       <x:c r="C26" t="str">
-        <x:v>For outer row 0, the inner loop prints `0` three times on one line. The empty `print()` starts a new line. The second outer pass prints `1` three times. The layout is `000` above `111`.</x:v>
+        <x:v>The outer loop creates rows 1, 2, and 3. On each row, the inner range ends at `row + 1`, so it prints the numbers from 1 through the current row. The resulting pattern is `1`, then `12`, then `123`.</x:v>
       </x:c>
       <x:c r="D26" t="n">
         <x:v>10</x:v>
@@ -1904,16 +1904,16 @@
       </x:c>
       <x:c r="L26"/>
       <x:c r="M26" t="str">
-        <x:v>`01` on each of three lines</x:v>
+        <x:v>`123` on each of three lines</x:v>
       </x:c>
       <x:c r="N26" t="str">
-        <x:v>`000` on line 1; `111` on line 2</x:v>
+        <x:v>`1` on line 1; `12` on line 2; `123` on line 3</x:v>
       </x:c>
       <x:c r="O26" t="str">
-        <x:v>`012` on each of two lines</x:v>
+        <x:v>`1` on line 1; `22` on line 2; `333` on line 3</x:v>
       </x:c>
       <x:c r="P26" t="str">
-        <x:v>`000111` on one line</x:v>
+        <x:v>`123` on a single line</x:v>
       </x:c>
       <x:c r="Q26" t="n">
         <x:v>2</x:v>
@@ -2374,18 +2374,17 @@
         <x:v>Python - MCQ - 4.2.24</x:v>
       </x:c>
       <x:c r="B35" t="str">
-        <x:v>A grid scan stops each row when it reaches column 3:
-```python
-for row in range(1, 4):
-    for column in range(1, 5):
-        if column == 3:
-            break
-        print(row, column)
-```
-How many pairs print, and does the outer loop stop?</x:v>
+        <x:v>A banner uses a descending `range()` to print a shrinking star pattern:
+```python
+for row in range(4, 0, -1):
+    for star in range(row):
+        print("*", end="")
+    print()
+```
+Which pattern is produced?</x:v>
       </x:c>
       <x:c r="C35" t="str">
-        <x:v>For each of the three rows, columns 1 and 2 print, then `break` exits only the inner loop at column 3. The outer loop continues with the next row. That produces 3 × 2 = 6 pairs.</x:v>
+        <x:v>The outer loop supplies 4, 3, 2, then 1. The inner loop prints exactly `row` stars before the empty `print()` starts the next line. Therefore the rows shrink from four stars to one star.</x:v>
       </x:c>
       <x:c r="D35" t="n">
         <x:v>10</x:v>
@@ -2413,16 +2412,16 @@
       </x:c>
       <x:c r="L35"/>
       <x:c r="M35" t="str">
-        <x:v>2 pairs; both loops stop at column 3</x:v>
+        <x:v>One row containing ten stars</x:v>
       </x:c>
       <x:c r="N35" t="str">
-        <x:v>3 pairs; one pair prints per row</x:v>
+        <x:v>Rows containing 1, 2, 3, then 4 stars</x:v>
       </x:c>
       <x:c r="O35" t="str">
-        <x:v>6 pairs; only the inner loop stops each time</x:v>
+        <x:v>Rows containing 4, 3, 2, then 1 star</x:v>
       </x:c>
       <x:c r="P35" t="str">
-        <x:v>12 pairs; `break` has no effect in nested loops</x:v>
+        <x:v>Four rows containing four stars each</x:v>
       </x:c>
       <x:c r="Q35" t="n">
         <x:v>3</x:v>
@@ -2724,21 +2723,19 @@
         <x:v>Python - MCQ - 4.2.30</x:v>
       </x:c>
       <x:c r="B41" t="str">
-        <x:v>Two versions each print six `X` characters:
-```python
-# Version A
-for row in range(2):
-    for column in range(3):
-        print("X", end="")
+        <x:v>A display prints spaces before stars to align a three-row pattern:
+```python
+for row in range(1, 4):
+    for space in range(3 - row):
+        print(" ", end="")
+    for star in range(row):
+        print("*", end="")
     print()
-# Version B
-for item in range(6):
-    print("X", end="")
-```
-Are their visible results equivalent?</x:v>
+```
+Which description matches the output?</x:v>
       </x:c>
       <x:c r="C41" t="str">
-        <x:v>Both versions print six characters, but Version A uses the outer loop to create two lines of three `X` characters. Version B never prints a newline, so all six appear on one line. Equal counts do not make the layouts equivalent.</x:v>
+        <x:v>The first inner loop prints 2, 1, then 0 leading spaces, while the second prints 1, 2, then 3 stars. The decreasing indentation keeps the final star of every row aligned, producing a right-aligned growing triangle.</x:v>
       </x:c>
       <x:c r="D41" t="n">
         <x:v>10</x:v>
@@ -2766,16 +2763,16 @@
       </x:c>
       <x:c r="L41"/>
       <x:c r="M41" t="str">
-        <x:v>Yes; any six printed characters have the same layout</x:v>
+        <x:v>A left-aligned triangle with 1, 2, then 3 stars</x:v>
       </x:c>
       <x:c r="N41" t="str">
-        <x:v>Yes; both create two rows of three</x:v>
+        <x:v>A shrinking triangle with 3, 2, then 1 star</x:v>
       </x:c>
       <x:c r="O41" t="str">
-        <x:v>No; Version A prints only three characters</x:v>
+        <x:v>A 3 by 3 square with spaces after each star</x:v>
       </x:c>
       <x:c r="P41" t="str">
-        <x:v>No; A makes two rows and B makes one line</x:v>
+        <x:v>A right-aligned triangle with 1, 2, then 3 stars</x:v>
       </x:c>
       <x:c r="Q41" t="n">
         <x:v>4</x:v>

</xml_diff>